<commit_message>
Remove surplus nomadic tab
</commit_message>
<xml_diff>
--- a/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
+++ b/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\git\nomadic\src\nomadic\start\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4A8232-E2E3-4D4E-9B71-C4B2CF93D9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00BB107C-677E-4659-B7D2-C2207D8E71B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="46260" windowHeight="23220" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="27288" windowHeight="15444" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="2" r:id="rId1"/>
     <sheet name="Gel" sheetId="8" r:id="rId2"/>
-    <sheet name="nomadic" sheetId="6" state="hidden" r:id="rId3"/>
-    <sheet name="options" sheetId="7" state="hidden" r:id="rId4"/>
-    <sheet name="Instructions" sheetId="9" r:id="rId5"/>
+    <sheet name="options" sheetId="7" state="hidden" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="9" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="Post_PCR_DNA_threshold_ngul">options!$B$1</definedName>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
   <si>
     <t>(YYYY-MM-DD)</t>
   </si>
@@ -345,12 +344,6 @@
     <t>H12</t>
   </si>
   <si>
-    <t>sample_id</t>
-  </si>
-  <si>
-    <t>barcode</t>
-  </si>
-  <si>
     <t>Sample Type</t>
   </si>
   <si>
@@ -370,9 +363,6 @@
   </si>
   <si>
     <t>Batch:</t>
-  </si>
-  <si>
-    <t>post_pcr_dna_conc_ngul</t>
   </si>
   <si>
     <t>Post PCR DNA threshold (ng / µl)</t>
@@ -943,20 +933,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -969,9 +946,22 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -982,7 +972,7 @@
     <cellStyle name="Normal 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
     <cellStyle name="Normal 4" xfId="5" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="18">
     <dxf>
       <fill>
         <patternFill>
@@ -1027,15 +1017,6 @@
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1515,45 +1496,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tbl_SeqLib" displayName="tbl_SeqLib" ref="A9:I105" totalsRowShown="0" headerRowDxfId="20" dataDxfId="18" headerRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tbl_SeqLib" displayName="tbl_SeqLib" ref="A9:I105" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16">
   <tableColumns count="9">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Well" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Sample ID" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Barcode" dataDxfId="15"/>
-    <tableColumn id="26" xr3:uid="{CDAB9BF6-0E65-46A9-85EA-6751A98F15D6}" name="Sample Type" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PCR [DNA] (ng / µl)" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{AB50544D-BD3B-4916-A4E2-114385DE79D0}" name="Duplicate Barcode" dataDxfId="12">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Well" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Sample ID" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Barcode" dataDxfId="12"/>
+    <tableColumn id="26" xr3:uid="{CDAB9BF6-0E65-46A9-85EA-6751A98F15D6}" name="Sample Type" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PCR [DNA] (ng / µl)" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{AB50544D-BD3B-4916-A4E2-114385DE79D0}" name="Duplicate Barcode" dataDxfId="9">
       <calculatedColumnFormula>IF(COUNTIF(tbl_SeqLib[Barcode],tbl_SeqLib[[#This Row],[Barcode]])&gt;1,TRUE,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A39E7F3C-2D21-4BE2-8657-FF30B6EAE695}" name="Valid Entry" dataDxfId="11">
+    <tableColumn id="6" xr3:uid="{A39E7F3C-2D21-4BE2-8657-FF30B6EAE695}" name="Valid Entry" dataDxfId="8">
       <calculatedColumnFormula>IF(OR(ISBLANK(tbl_SeqLib[[#This Row],[Sample ID]]),ISBLANK(tbl_SeqLib[[#This Row],[Barcode]]),ISBLANK(tbl_SeqLib[[#This Row],[Sample Type]])),FALSE, TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{1729EBF8-66DF-4C30-A401-833B6EC9ECE7}" name="Data entered" dataDxfId="10">
+    <tableColumn id="7" xr3:uid="{1729EBF8-66DF-4C30-A401-833B6EC9ECE7}" name="Data entered" dataDxfId="7">
       <calculatedColumnFormula>IF(AND(ISBLANK(tbl_SeqLib[[#This Row],[Sample ID]]),ISBLANK(tbl_SeqLib[[#This Row],[Sample Type]]),ISBLANK(tbl_SeqLib[[#This Row],[PCR '[DNA'] (ng / µl)]])),FALSE,TRUE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{CB344B8B-24D4-4560-B5B0-D807A540F109}" name="Errors" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{CB344B8B-24D4-4560-B5B0-D807A540F109}" name="Errors" dataDxfId="6">
       <calculatedColumnFormula>IF(tbl_SeqLib[[#This Row],[Duplicate Barcode]],"DUPLICATE BARCODE",IF(AND(tbl_SeqLib[[#This Row],[Data entered]],NOT(tbl_SeqLib[[#This Row],[Valid Entry]])),"Incomplete Entry",""))</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tbl_nomadic" displayName="tbl_nomadic" ref="A1:D97" totalsRowShown="0">
-  <autoFilter ref="A1:D97" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="sample_id">
-      <calculatedColumnFormula>IF(Library!G10,Library!B10,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="9" xr3:uid="{98E62512-61AC-41C9-8930-37E9E6964CA3}" name="sample_type" dataDxfId="8">
-      <calculatedColumnFormula>IF(Library!G10,Library!D10,"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="barcode" dataDxfId="7">
-      <calculatedColumnFormula>IF(Library!G10,CONCATENATE("barcode",TEXT(Library!C10,"00")),"")</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{1FDA51E1-A0B8-4EA2-9C5A-4746ACED2260}" name="post_pcr_dna_conc_ngul" dataDxfId="6">
-      <calculatedColumnFormula>IF(AND(Library!G10,NOT(ISBLANK(Library!E10))),Library!E10,"")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1753,25 +1713,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
-        <v>107</v>
-      </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
+      <c r="A1" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
-        <v>126</v>
-      </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="A2" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" s="38"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
       <c r="E2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1780,67 +1740,67 @@
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="38"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
-        <v>106</v>
-      </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
       <c r="E4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="38" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
+      <c r="A6" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="42"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
       <c r="E6" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="42" t="str">
+      <c r="B7" s="43"/>
+      <c r="C7" s="46" t="str">
         <f>IF(OR(ISBLANK(C2),ISBLANK(C3),ISBLANK(C4), ISBLANK(C5), ISBLANK(C6)),"",CONCATENATE(C2,"_",C3,TEXT(C5,"000"),"_",C4,"_Batch",C6))</f>
         <v/>
       </c>
-      <c r="D7" s="42"/>
+      <c r="D7" s="46"/>
       <c r="E7" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -1854,28 +1814,28 @@
         <v>2</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>3</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -4583,6 +4543,12 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:I1"/>
@@ -4590,12 +4556,6 @@
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="B10:E105">
@@ -4687,1771 +4647,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FFFF0000"/>
-  </sheetPr>
-  <dimension ref="A1:D97"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.19921875" customWidth="1"/>
-    <col min="2" max="3" width="13.69921875" customWidth="1"/>
-    <col min="4" max="4" width="30.59765625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="str">
-        <f>IF(Library!G10,Library!B10,"")</f>
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <f>IF(Library!G10,Library!D10,"")</f>
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <f>IF(Library!G10,CONCATENATE("barcode",TEXT(Library!C10,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <f>IF(AND(Library!G10,NOT(ISBLANK(Library!E10))),Library!E10,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="str">
-        <f>IF(Library!G11,Library!B11,"")</f>
-        <v/>
-      </c>
-      <c r="B3" t="str">
-        <f>IF(Library!G11,Library!D11,"")</f>
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <f>IF(Library!G11,CONCATENATE("barcode",TEXT(Library!C11,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <f>IF(AND(Library!G11,NOT(ISBLANK(Library!E11))),Library!E11,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="str">
-        <f>IF(Library!G12,Library!B12,"")</f>
-        <v/>
-      </c>
-      <c r="B4" t="str">
-        <f>IF(Library!G12,Library!D12,"")</f>
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <f>IF(Library!G12,CONCATENATE("barcode",TEXT(Library!C12,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <f>IF(AND(Library!G12,NOT(ISBLANK(Library!E12))),Library!E12,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="str">
-        <f>IF(Library!G13,Library!B13,"")</f>
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <f>IF(Library!G13,Library!D13,"")</f>
-        <v/>
-      </c>
-      <c r="C5" t="str">
-        <f>IF(Library!G13,CONCATENATE("barcode",TEXT(Library!C13,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <f>IF(AND(Library!G13,NOT(ISBLANK(Library!E13))),Library!E13,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="str">
-        <f>IF(Library!G14,Library!B14,"")</f>
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <f>IF(Library!G14,Library!D14,"")</f>
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <f>IF(Library!G14,CONCATENATE("barcode",TEXT(Library!C14,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <f>IF(AND(Library!G14,NOT(ISBLANK(Library!E14))),Library!E14,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="str">
-        <f>IF(Library!G15,Library!B15,"")</f>
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <f>IF(Library!G15,Library!D15,"")</f>
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <f>IF(Library!G15,CONCATENATE("barcode",TEXT(Library!C15,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <f>IF(AND(Library!G15,NOT(ISBLANK(Library!E15))),Library!E15,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="str">
-        <f>IF(Library!G16,Library!B16,"")</f>
-        <v/>
-      </c>
-      <c r="B8" t="str">
-        <f>IF(Library!G16,Library!D16,"")</f>
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <f>IF(Library!G16,CONCATENATE("barcode",TEXT(Library!C16,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <f>IF(AND(Library!G16,NOT(ISBLANK(Library!E16))),Library!E16,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="str">
-        <f>IF(Library!G17,Library!B17,"")</f>
-        <v/>
-      </c>
-      <c r="B9" t="str">
-        <f>IF(Library!G17,Library!D17,"")</f>
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <f>IF(Library!G17,CONCATENATE("barcode",TEXT(Library!C17,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <f>IF(AND(Library!G17,NOT(ISBLANK(Library!E17))),Library!E17,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="str">
-        <f>IF(Library!G18,Library!B18,"")</f>
-        <v/>
-      </c>
-      <c r="B10" t="str">
-        <f>IF(Library!G18,Library!D18,"")</f>
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <f>IF(Library!G18,CONCATENATE("barcode",TEXT(Library!C18,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <f>IF(AND(Library!G18,NOT(ISBLANK(Library!E18))),Library!E18,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="str">
-        <f>IF(Library!G19,Library!B19,"")</f>
-        <v/>
-      </c>
-      <c r="B11" t="str">
-        <f>IF(Library!G19,Library!D19,"")</f>
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <f>IF(Library!G19,CONCATENATE("barcode",TEXT(Library!C19,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <f>IF(AND(Library!G19,NOT(ISBLANK(Library!E19))),Library!E19,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="str">
-        <f>IF(Library!G20,Library!B20,"")</f>
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <f>IF(Library!G20,Library!D20,"")</f>
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <f>IF(Library!G20,CONCATENATE("barcode",TEXT(Library!C20,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D12" t="str">
-        <f>IF(AND(Library!G20,NOT(ISBLANK(Library!E20))),Library!E20,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="str">
-        <f>IF(Library!G21,Library!B21,"")</f>
-        <v/>
-      </c>
-      <c r="B13" t="str">
-        <f>IF(Library!G21,Library!D21,"")</f>
-        <v/>
-      </c>
-      <c r="C13" t="str">
-        <f>IF(Library!G21,CONCATENATE("barcode",TEXT(Library!C21,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <f>IF(AND(Library!G21,NOT(ISBLANK(Library!E21))),Library!E21,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="str">
-        <f>IF(Library!G22,Library!B22,"")</f>
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <f>IF(Library!G22,Library!D22,"")</f>
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <f>IF(Library!G22,CONCATENATE("barcode",TEXT(Library!C22,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <f>IF(AND(Library!G22,NOT(ISBLANK(Library!E22))),Library!E22,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="str">
-        <f>IF(Library!G23,Library!B23,"")</f>
-        <v/>
-      </c>
-      <c r="B15" t="str">
-        <f>IF(Library!G23,Library!D23,"")</f>
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <f>IF(Library!G23,CONCATENATE("barcode",TEXT(Library!C23,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <f>IF(AND(Library!G23,NOT(ISBLANK(Library!E23))),Library!E23,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" t="str">
-        <f>IF(Library!G24,Library!B24,"")</f>
-        <v/>
-      </c>
-      <c r="B16" t="str">
-        <f>IF(Library!G24,Library!D24,"")</f>
-        <v/>
-      </c>
-      <c r="C16" t="str">
-        <f>IF(Library!G24,CONCATENATE("barcode",TEXT(Library!C24,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <f>IF(AND(Library!G24,NOT(ISBLANK(Library!E24))),Library!E24,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="str">
-        <f>IF(Library!G25,Library!B25,"")</f>
-        <v/>
-      </c>
-      <c r="B17" t="str">
-        <f>IF(Library!G25,Library!D25,"")</f>
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <f>IF(Library!G25,CONCATENATE("barcode",TEXT(Library!C25,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <f>IF(AND(Library!G25,NOT(ISBLANK(Library!E25))),Library!E25,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" t="str">
-        <f>IF(Library!G26,Library!B26,"")</f>
-        <v/>
-      </c>
-      <c r="B18" t="str">
-        <f>IF(Library!G26,Library!D26,"")</f>
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <f>IF(Library!G26,CONCATENATE("barcode",TEXT(Library!C26,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <f>IF(AND(Library!G26,NOT(ISBLANK(Library!E26))),Library!E26,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="str">
-        <f>IF(Library!G27,Library!B27,"")</f>
-        <v/>
-      </c>
-      <c r="B19" t="str">
-        <f>IF(Library!G27,Library!D27,"")</f>
-        <v/>
-      </c>
-      <c r="C19" t="str">
-        <f>IF(Library!G27,CONCATENATE("barcode",TEXT(Library!C27,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <f>IF(AND(Library!G27,NOT(ISBLANK(Library!E27))),Library!E27,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="str">
-        <f>IF(Library!G28,Library!B28,"")</f>
-        <v/>
-      </c>
-      <c r="B20" t="str">
-        <f>IF(Library!G28,Library!D28,"")</f>
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <f>IF(Library!G28,CONCATENATE("barcode",TEXT(Library!C28,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D20" t="str">
-        <f>IF(AND(Library!G28,NOT(ISBLANK(Library!E28))),Library!E28,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="str">
-        <f>IF(Library!G29,Library!B29,"")</f>
-        <v/>
-      </c>
-      <c r="B21" t="str">
-        <f>IF(Library!G29,Library!D29,"")</f>
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <f>IF(Library!G29,CONCATENATE("barcode",TEXT(Library!C29,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <f>IF(AND(Library!G29,NOT(ISBLANK(Library!E29))),Library!E29,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="str">
-        <f>IF(Library!G30,Library!B30,"")</f>
-        <v/>
-      </c>
-      <c r="B22" t="str">
-        <f>IF(Library!G30,Library!D30,"")</f>
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <f>IF(Library!G30,CONCATENATE("barcode",TEXT(Library!C30,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D22" t="str">
-        <f>IF(AND(Library!G30,NOT(ISBLANK(Library!E30))),Library!E30,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="str">
-        <f>IF(Library!G31,Library!B31,"")</f>
-        <v/>
-      </c>
-      <c r="B23" t="str">
-        <f>IF(Library!G31,Library!D31,"")</f>
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <f>IF(Library!G31,CONCATENATE("barcode",TEXT(Library!C31,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D23" t="str">
-        <f>IF(AND(Library!G31,NOT(ISBLANK(Library!E31))),Library!E31,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="str">
-        <f>IF(Library!G32,Library!B32,"")</f>
-        <v/>
-      </c>
-      <c r="B24" t="str">
-        <f>IF(Library!G32,Library!D32,"")</f>
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <f>IF(Library!G32,CONCATENATE("barcode",TEXT(Library!C32,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D24" t="str">
-        <f>IF(AND(Library!G32,NOT(ISBLANK(Library!E32))),Library!E32,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" t="str">
-        <f>IF(Library!G33,Library!B33,"")</f>
-        <v/>
-      </c>
-      <c r="B25" t="str">
-        <f>IF(Library!G33,Library!D33,"")</f>
-        <v/>
-      </c>
-      <c r="C25" t="str">
-        <f>IF(Library!G33,CONCATENATE("barcode",TEXT(Library!C33,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D25" t="str">
-        <f>IF(AND(Library!G33,NOT(ISBLANK(Library!E33))),Library!E33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" t="str">
-        <f>IF(Library!G34,Library!B34,"")</f>
-        <v/>
-      </c>
-      <c r="B26" t="str">
-        <f>IF(Library!G34,Library!D34,"")</f>
-        <v/>
-      </c>
-      <c r="C26" t="str">
-        <f>IF(Library!G34,CONCATENATE("barcode",TEXT(Library!C34,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D26" t="str">
-        <f>IF(AND(Library!G34,NOT(ISBLANK(Library!E34))),Library!E34,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" t="str">
-        <f>IF(Library!G35,Library!B35,"")</f>
-        <v/>
-      </c>
-      <c r="B27" t="str">
-        <f>IF(Library!G35,Library!D35,"")</f>
-        <v/>
-      </c>
-      <c r="C27" t="str">
-        <f>IF(Library!G35,CONCATENATE("barcode",TEXT(Library!C35,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D27" t="str">
-        <f>IF(AND(Library!G35,NOT(ISBLANK(Library!E35))),Library!E35,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" t="str">
-        <f>IF(Library!G36,Library!B36,"")</f>
-        <v/>
-      </c>
-      <c r="B28" t="str">
-        <f>IF(Library!G36,Library!D36,"")</f>
-        <v/>
-      </c>
-      <c r="C28" t="str">
-        <f>IF(Library!G36,CONCATENATE("barcode",TEXT(Library!C36,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D28" t="str">
-        <f>IF(AND(Library!G36,NOT(ISBLANK(Library!E36))),Library!E36,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" t="str">
-        <f>IF(Library!G37,Library!B37,"")</f>
-        <v/>
-      </c>
-      <c r="B29" t="str">
-        <f>IF(Library!G37,Library!D37,"")</f>
-        <v/>
-      </c>
-      <c r="C29" t="str">
-        <f>IF(Library!G37,CONCATENATE("barcode",TEXT(Library!C37,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D29" t="str">
-        <f>IF(AND(Library!G37,NOT(ISBLANK(Library!E37))),Library!E37,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" t="str">
-        <f>IF(Library!G38,Library!B38,"")</f>
-        <v/>
-      </c>
-      <c r="B30" t="str">
-        <f>IF(Library!G38,Library!D38,"")</f>
-        <v/>
-      </c>
-      <c r="C30" t="str">
-        <f>IF(Library!G38,CONCATENATE("barcode",TEXT(Library!C38,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D30" t="str">
-        <f>IF(AND(Library!G38,NOT(ISBLANK(Library!E38))),Library!E38,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" t="str">
-        <f>IF(Library!G39,Library!B39,"")</f>
-        <v/>
-      </c>
-      <c r="B31" t="str">
-        <f>IF(Library!G39,Library!D39,"")</f>
-        <v/>
-      </c>
-      <c r="C31" t="str">
-        <f>IF(Library!G39,CONCATENATE("barcode",TEXT(Library!C39,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D31" t="str">
-        <f>IF(AND(Library!G39,NOT(ISBLANK(Library!E39))),Library!E39,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" t="str">
-        <f>IF(Library!G40,Library!B40,"")</f>
-        <v/>
-      </c>
-      <c r="B32" t="str">
-        <f>IF(Library!G40,Library!D40,"")</f>
-        <v/>
-      </c>
-      <c r="C32" t="str">
-        <f>IF(Library!G40,CONCATENATE("barcode",TEXT(Library!C40,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D32" t="str">
-        <f>IF(AND(Library!G40,NOT(ISBLANK(Library!E40))),Library!E40,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" t="str">
-        <f>IF(Library!G41,Library!B41,"")</f>
-        <v/>
-      </c>
-      <c r="B33" t="str">
-        <f>IF(Library!G41,Library!D41,"")</f>
-        <v/>
-      </c>
-      <c r="C33" t="str">
-        <f>IF(Library!G41,CONCATENATE("barcode",TEXT(Library!C41,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D33" t="str">
-        <f>IF(AND(Library!G41,NOT(ISBLANK(Library!E41))),Library!E41,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" t="str">
-        <f>IF(Library!G42,Library!B42,"")</f>
-        <v/>
-      </c>
-      <c r="B34" t="str">
-        <f>IF(Library!G42,Library!D42,"")</f>
-        <v/>
-      </c>
-      <c r="C34" t="str">
-        <f>IF(Library!G42,CONCATENATE("barcode",TEXT(Library!C42,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D34" t="str">
-        <f>IF(AND(Library!G42,NOT(ISBLANK(Library!E42))),Library!E42,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" t="str">
-        <f>IF(Library!G43,Library!B43,"")</f>
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <f>IF(Library!G43,Library!D43,"")</f>
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <f>IF(Library!G43,CONCATENATE("barcode",TEXT(Library!C43,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D35" t="str">
-        <f>IF(AND(Library!G43,NOT(ISBLANK(Library!E43))),Library!E43,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" t="str">
-        <f>IF(Library!G44,Library!B44,"")</f>
-        <v/>
-      </c>
-      <c r="B36" t="str">
-        <f>IF(Library!G44,Library!D44,"")</f>
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <f>IF(Library!G44,CONCATENATE("barcode",TEXT(Library!C44,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D36" t="str">
-        <f>IF(AND(Library!G44,NOT(ISBLANK(Library!E44))),Library!E44,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" t="str">
-        <f>IF(Library!G45,Library!B45,"")</f>
-        <v/>
-      </c>
-      <c r="B37" t="str">
-        <f>IF(Library!G45,Library!D45,"")</f>
-        <v/>
-      </c>
-      <c r="C37" t="str">
-        <f>IF(Library!G45,CONCATENATE("barcode",TEXT(Library!C45,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D37" t="str">
-        <f>IF(AND(Library!G45,NOT(ISBLANK(Library!E45))),Library!E45,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" t="str">
-        <f>IF(Library!G46,Library!B46,"")</f>
-        <v/>
-      </c>
-      <c r="B38" t="str">
-        <f>IF(Library!G46,Library!D46,"")</f>
-        <v/>
-      </c>
-      <c r="C38" t="str">
-        <f>IF(Library!G46,CONCATENATE("barcode",TEXT(Library!C46,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D38" t="str">
-        <f>IF(AND(Library!G46,NOT(ISBLANK(Library!E46))),Library!E46,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" t="str">
-        <f>IF(Library!G47,Library!B47,"")</f>
-        <v/>
-      </c>
-      <c r="B39" t="str">
-        <f>IF(Library!G47,Library!D47,"")</f>
-        <v/>
-      </c>
-      <c r="C39" t="str">
-        <f>IF(Library!G47,CONCATENATE("barcode",TEXT(Library!C47,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D39" t="str">
-        <f>IF(AND(Library!G47,NOT(ISBLANK(Library!E47))),Library!E47,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" t="str">
-        <f>IF(Library!G48,Library!B48,"")</f>
-        <v/>
-      </c>
-      <c r="B40" t="str">
-        <f>IF(Library!G48,Library!D48,"")</f>
-        <v/>
-      </c>
-      <c r="C40" t="str">
-        <f>IF(Library!G48,CONCATENATE("barcode",TEXT(Library!C48,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D40" t="str">
-        <f>IF(AND(Library!G48,NOT(ISBLANK(Library!E48))),Library!E48,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" t="str">
-        <f>IF(Library!G49,Library!B49,"")</f>
-        <v/>
-      </c>
-      <c r="B41" t="str">
-        <f>IF(Library!G49,Library!D49,"")</f>
-        <v/>
-      </c>
-      <c r="C41" t="str">
-        <f>IF(Library!G49,CONCATENATE("barcode",TEXT(Library!C49,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D41" t="str">
-        <f>IF(AND(Library!G49,NOT(ISBLANK(Library!E49))),Library!E49,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" t="str">
-        <f>IF(Library!G50,Library!B50,"")</f>
-        <v/>
-      </c>
-      <c r="B42" t="str">
-        <f>IF(Library!G50,Library!D50,"")</f>
-        <v/>
-      </c>
-      <c r="C42" t="str">
-        <f>IF(Library!G50,CONCATENATE("barcode",TEXT(Library!C50,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D42" t="str">
-        <f>IF(AND(Library!G50,NOT(ISBLANK(Library!E50))),Library!E50,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" t="str">
-        <f>IF(Library!G51,Library!B51,"")</f>
-        <v/>
-      </c>
-      <c r="B43" t="str">
-        <f>IF(Library!G51,Library!D51,"")</f>
-        <v/>
-      </c>
-      <c r="C43" t="str">
-        <f>IF(Library!G51,CONCATENATE("barcode",TEXT(Library!C51,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D43" t="str">
-        <f>IF(AND(Library!G51,NOT(ISBLANK(Library!E51))),Library!E51,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" t="str">
-        <f>IF(Library!G52,Library!B52,"")</f>
-        <v/>
-      </c>
-      <c r="B44" t="str">
-        <f>IF(Library!G52,Library!D52,"")</f>
-        <v/>
-      </c>
-      <c r="C44" t="str">
-        <f>IF(Library!G52,CONCATENATE("barcode",TEXT(Library!C52,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D44" t="str">
-        <f>IF(AND(Library!G52,NOT(ISBLANK(Library!E52))),Library!E52,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" t="str">
-        <f>IF(Library!G53,Library!B53,"")</f>
-        <v/>
-      </c>
-      <c r="B45" t="str">
-        <f>IF(Library!G53,Library!D53,"")</f>
-        <v/>
-      </c>
-      <c r="C45" t="str">
-        <f>IF(Library!G53,CONCATENATE("barcode",TEXT(Library!C53,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D45" t="str">
-        <f>IF(AND(Library!G53,NOT(ISBLANK(Library!E53))),Library!E53,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" t="str">
-        <f>IF(Library!G54,Library!B54,"")</f>
-        <v/>
-      </c>
-      <c r="B46" t="str">
-        <f>IF(Library!G54,Library!D54,"")</f>
-        <v/>
-      </c>
-      <c r="C46" t="str">
-        <f>IF(Library!G54,CONCATENATE("barcode",TEXT(Library!C54,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D46" t="str">
-        <f>IF(AND(Library!G54,NOT(ISBLANK(Library!E54))),Library!E54,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" t="str">
-        <f>IF(Library!G55,Library!B55,"")</f>
-        <v/>
-      </c>
-      <c r="B47" t="str">
-        <f>IF(Library!G55,Library!D55,"")</f>
-        <v/>
-      </c>
-      <c r="C47" t="str">
-        <f>IF(Library!G55,CONCATENATE("barcode",TEXT(Library!C55,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D47" t="str">
-        <f>IF(AND(Library!G55,NOT(ISBLANK(Library!E55))),Library!E55,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A48" t="str">
-        <f>IF(Library!G56,Library!B56,"")</f>
-        <v/>
-      </c>
-      <c r="B48" t="str">
-        <f>IF(Library!G56,Library!D56,"")</f>
-        <v/>
-      </c>
-      <c r="C48" t="str">
-        <f>IF(Library!G56,CONCATENATE("barcode",TEXT(Library!C56,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D48" t="str">
-        <f>IF(AND(Library!G56,NOT(ISBLANK(Library!E56))),Library!E56,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" t="str">
-        <f>IF(Library!G57,Library!B57,"")</f>
-        <v/>
-      </c>
-      <c r="B49" t="str">
-        <f>IF(Library!G57,Library!D57,"")</f>
-        <v/>
-      </c>
-      <c r="C49" t="str">
-        <f>IF(Library!G57,CONCATENATE("barcode",TEXT(Library!C57,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D49" t="str">
-        <f>IF(AND(Library!G57,NOT(ISBLANK(Library!E57))),Library!E57,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A50" t="str">
-        <f>IF(Library!G58,Library!B58,"")</f>
-        <v/>
-      </c>
-      <c r="B50" t="str">
-        <f>IF(Library!G58,Library!D58,"")</f>
-        <v/>
-      </c>
-      <c r="C50" t="str">
-        <f>IF(Library!G58,CONCATENATE("barcode",TEXT(Library!C58,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D50" t="str">
-        <f>IF(AND(Library!G58,NOT(ISBLANK(Library!E58))),Library!E58,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A51" t="str">
-        <f>IF(Library!G59,Library!B59,"")</f>
-        <v/>
-      </c>
-      <c r="B51" t="str">
-        <f>IF(Library!G59,Library!D59,"")</f>
-        <v/>
-      </c>
-      <c r="C51" t="str">
-        <f>IF(Library!G59,CONCATENATE("barcode",TEXT(Library!C59,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D51" t="str">
-        <f>IF(AND(Library!G59,NOT(ISBLANK(Library!E59))),Library!E59,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" t="str">
-        <f>IF(Library!G60,Library!B60,"")</f>
-        <v/>
-      </c>
-      <c r="B52" t="str">
-        <f>IF(Library!G60,Library!D60,"")</f>
-        <v/>
-      </c>
-      <c r="C52" t="str">
-        <f>IF(Library!G60,CONCATENATE("barcode",TEXT(Library!C60,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D52" t="str">
-        <f>IF(AND(Library!G60,NOT(ISBLANK(Library!E60))),Library!E60,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" t="str">
-        <f>IF(Library!G61,Library!B61,"")</f>
-        <v/>
-      </c>
-      <c r="B53" t="str">
-        <f>IF(Library!G61,Library!D61,"")</f>
-        <v/>
-      </c>
-      <c r="C53" t="str">
-        <f>IF(Library!G61,CONCATENATE("barcode",TEXT(Library!C61,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D53" t="str">
-        <f>IF(AND(Library!G61,NOT(ISBLANK(Library!E61))),Library!E61,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" t="str">
-        <f>IF(Library!G62,Library!B62,"")</f>
-        <v/>
-      </c>
-      <c r="B54" t="str">
-        <f>IF(Library!G62,Library!D62,"")</f>
-        <v/>
-      </c>
-      <c r="C54" t="str">
-        <f>IF(Library!G62,CONCATENATE("barcode",TEXT(Library!C62,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D54" t="str">
-        <f>IF(AND(Library!G62,NOT(ISBLANK(Library!E62))),Library!E62,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" t="str">
-        <f>IF(Library!G63,Library!B63,"")</f>
-        <v/>
-      </c>
-      <c r="B55" t="str">
-        <f>IF(Library!G63,Library!D63,"")</f>
-        <v/>
-      </c>
-      <c r="C55" t="str">
-        <f>IF(Library!G63,CONCATENATE("barcode",TEXT(Library!C63,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D55" t="str">
-        <f>IF(AND(Library!G63,NOT(ISBLANK(Library!E63))),Library!E63,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" t="str">
-        <f>IF(Library!G64,Library!B64,"")</f>
-        <v/>
-      </c>
-      <c r="B56" t="str">
-        <f>IF(Library!G64,Library!D64,"")</f>
-        <v/>
-      </c>
-      <c r="C56" t="str">
-        <f>IF(Library!G64,CONCATENATE("barcode",TEXT(Library!C64,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D56" t="str">
-        <f>IF(AND(Library!G64,NOT(ISBLANK(Library!E64))),Library!E64,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" t="str">
-        <f>IF(Library!G65,Library!B65,"")</f>
-        <v/>
-      </c>
-      <c r="B57" t="str">
-        <f>IF(Library!G65,Library!D65,"")</f>
-        <v/>
-      </c>
-      <c r="C57" t="str">
-        <f>IF(Library!G65,CONCATENATE("barcode",TEXT(Library!C65,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D57" t="str">
-        <f>IF(AND(Library!G65,NOT(ISBLANK(Library!E65))),Library!E65,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" t="str">
-        <f>IF(Library!G66,Library!B66,"")</f>
-        <v/>
-      </c>
-      <c r="B58" t="str">
-        <f>IF(Library!G66,Library!D66,"")</f>
-        <v/>
-      </c>
-      <c r="C58" t="str">
-        <f>IF(Library!G66,CONCATENATE("barcode",TEXT(Library!C66,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D58" t="str">
-        <f>IF(AND(Library!G66,NOT(ISBLANK(Library!E66))),Library!E66,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" t="str">
-        <f>IF(Library!G67,Library!B67,"")</f>
-        <v/>
-      </c>
-      <c r="B59" t="str">
-        <f>IF(Library!G67,Library!D67,"")</f>
-        <v/>
-      </c>
-      <c r="C59" t="str">
-        <f>IF(Library!G67,CONCATENATE("barcode",TEXT(Library!C67,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D59" t="str">
-        <f>IF(AND(Library!G67,NOT(ISBLANK(Library!E67))),Library!E67,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" t="str">
-        <f>IF(Library!G68,Library!B68,"")</f>
-        <v/>
-      </c>
-      <c r="B60" t="str">
-        <f>IF(Library!G68,Library!D68,"")</f>
-        <v/>
-      </c>
-      <c r="C60" t="str">
-        <f>IF(Library!G68,CONCATENATE("barcode",TEXT(Library!C68,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D60" t="str">
-        <f>IF(AND(Library!G68,NOT(ISBLANK(Library!E68))),Library!E68,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" t="str">
-        <f>IF(Library!G69,Library!B69,"")</f>
-        <v/>
-      </c>
-      <c r="B61" t="str">
-        <f>IF(Library!G69,Library!D69,"")</f>
-        <v/>
-      </c>
-      <c r="C61" t="str">
-        <f>IF(Library!G69,CONCATENATE("barcode",TEXT(Library!C69,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D61" t="str">
-        <f>IF(AND(Library!G69,NOT(ISBLANK(Library!E69))),Library!E69,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A62" t="str">
-        <f>IF(Library!G70,Library!B70,"")</f>
-        <v/>
-      </c>
-      <c r="B62" t="str">
-        <f>IF(Library!G70,Library!D70,"")</f>
-        <v/>
-      </c>
-      <c r="C62" t="str">
-        <f>IF(Library!G70,CONCATENATE("barcode",TEXT(Library!C70,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D62" t="str">
-        <f>IF(AND(Library!G70,NOT(ISBLANK(Library!E70))),Library!E70,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" t="str">
-        <f>IF(Library!G71,Library!B71,"")</f>
-        <v/>
-      </c>
-      <c r="B63" t="str">
-        <f>IF(Library!G71,Library!D71,"")</f>
-        <v/>
-      </c>
-      <c r="C63" t="str">
-        <f>IF(Library!G71,CONCATENATE("barcode",TEXT(Library!C71,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D63" t="str">
-        <f>IF(AND(Library!G71,NOT(ISBLANK(Library!E71))),Library!E71,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" t="str">
-        <f>IF(Library!G72,Library!B72,"")</f>
-        <v/>
-      </c>
-      <c r="B64" t="str">
-        <f>IF(Library!G72,Library!D72,"")</f>
-        <v/>
-      </c>
-      <c r="C64" t="str">
-        <f>IF(Library!G72,CONCATENATE("barcode",TEXT(Library!C72,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D64" t="str">
-        <f>IF(AND(Library!G72,NOT(ISBLANK(Library!E72))),Library!E72,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" t="str">
-        <f>IF(Library!G73,Library!B73,"")</f>
-        <v/>
-      </c>
-      <c r="B65" t="str">
-        <f>IF(Library!G73,Library!D73,"")</f>
-        <v/>
-      </c>
-      <c r="C65" t="str">
-        <f>IF(Library!G73,CONCATENATE("barcode",TEXT(Library!C73,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D65" t="str">
-        <f>IF(AND(Library!G73,NOT(ISBLANK(Library!E73))),Library!E73,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" t="str">
-        <f>IF(Library!G74,Library!B74,"")</f>
-        <v/>
-      </c>
-      <c r="B66" t="str">
-        <f>IF(Library!G74,Library!D74,"")</f>
-        <v/>
-      </c>
-      <c r="C66" t="str">
-        <f>IF(Library!G74,CONCATENATE("barcode",TEXT(Library!C74,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D66" t="str">
-        <f>IF(AND(Library!G74,NOT(ISBLANK(Library!E74))),Library!E74,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" t="str">
-        <f>IF(Library!G75,Library!B75,"")</f>
-        <v/>
-      </c>
-      <c r="B67" t="str">
-        <f>IF(Library!G75,Library!D75,"")</f>
-        <v/>
-      </c>
-      <c r="C67" t="str">
-        <f>IF(Library!G75,CONCATENATE("barcode",TEXT(Library!C75,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D67" t="str">
-        <f>IF(AND(Library!G75,NOT(ISBLANK(Library!E75))),Library!E75,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" t="str">
-        <f>IF(Library!G76,Library!B76,"")</f>
-        <v/>
-      </c>
-      <c r="B68" t="str">
-        <f>IF(Library!G76,Library!D76,"")</f>
-        <v/>
-      </c>
-      <c r="C68" t="str">
-        <f>IF(Library!G76,CONCATENATE("barcode",TEXT(Library!C76,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D68" t="str">
-        <f>IF(AND(Library!G76,NOT(ISBLANK(Library!E76))),Library!E76,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" t="str">
-        <f>IF(Library!G77,Library!B77,"")</f>
-        <v/>
-      </c>
-      <c r="B69" t="str">
-        <f>IF(Library!G77,Library!D77,"")</f>
-        <v/>
-      </c>
-      <c r="C69" t="str">
-        <f>IF(Library!G77,CONCATENATE("barcode",TEXT(Library!C77,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D69" t="str">
-        <f>IF(AND(Library!G77,NOT(ISBLANK(Library!E77))),Library!E77,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" t="str">
-        <f>IF(Library!G78,Library!B78,"")</f>
-        <v/>
-      </c>
-      <c r="B70" t="str">
-        <f>IF(Library!G78,Library!D78,"")</f>
-        <v/>
-      </c>
-      <c r="C70" t="str">
-        <f>IF(Library!G78,CONCATENATE("barcode",TEXT(Library!C78,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D70" t="str">
-        <f>IF(AND(Library!G78,NOT(ISBLANK(Library!E78))),Library!E78,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" t="str">
-        <f>IF(Library!G79,Library!B79,"")</f>
-        <v/>
-      </c>
-      <c r="B71" t="str">
-        <f>IF(Library!G79,Library!D79,"")</f>
-        <v/>
-      </c>
-      <c r="C71" t="str">
-        <f>IF(Library!G79,CONCATENATE("barcode",TEXT(Library!C79,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D71" t="str">
-        <f>IF(AND(Library!G79,NOT(ISBLANK(Library!E79))),Library!E79,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" t="str">
-        <f>IF(Library!G80,Library!B80,"")</f>
-        <v/>
-      </c>
-      <c r="B72" t="str">
-        <f>IF(Library!G80,Library!D80,"")</f>
-        <v/>
-      </c>
-      <c r="C72" t="str">
-        <f>IF(Library!G80,CONCATENATE("barcode",TEXT(Library!C80,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D72" t="str">
-        <f>IF(AND(Library!G80,NOT(ISBLANK(Library!E80))),Library!E80,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" t="str">
-        <f>IF(Library!G81,Library!B81,"")</f>
-        <v/>
-      </c>
-      <c r="B73" t="str">
-        <f>IF(Library!G81,Library!D81,"")</f>
-        <v/>
-      </c>
-      <c r="C73" t="str">
-        <f>IF(Library!G81,CONCATENATE("barcode",TEXT(Library!C81,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D73" t="str">
-        <f>IF(AND(Library!G81,NOT(ISBLANK(Library!E81))),Library!E81,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" t="str">
-        <f>IF(Library!G82,Library!B82,"")</f>
-        <v/>
-      </c>
-      <c r="B74" t="str">
-        <f>IF(Library!G82,Library!D82,"")</f>
-        <v/>
-      </c>
-      <c r="C74" t="str">
-        <f>IF(Library!G82,CONCATENATE("barcode",TEXT(Library!C82,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D74" t="str">
-        <f>IF(AND(Library!G82,NOT(ISBLANK(Library!E82))),Library!E82,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" t="str">
-        <f>IF(Library!G83,Library!B83,"")</f>
-        <v/>
-      </c>
-      <c r="B75" t="str">
-        <f>IF(Library!G83,Library!D83,"")</f>
-        <v/>
-      </c>
-      <c r="C75" t="str">
-        <f>IF(Library!G83,CONCATENATE("barcode",TEXT(Library!C83,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D75" t="str">
-        <f>IF(AND(Library!G83,NOT(ISBLANK(Library!E83))),Library!E83,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" t="str">
-        <f>IF(Library!G84,Library!B84,"")</f>
-        <v/>
-      </c>
-      <c r="B76" t="str">
-        <f>IF(Library!G84,Library!D84,"")</f>
-        <v/>
-      </c>
-      <c r="C76" t="str">
-        <f>IF(Library!G84,CONCATENATE("barcode",TEXT(Library!C84,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D76" t="str">
-        <f>IF(AND(Library!G84,NOT(ISBLANK(Library!E84))),Library!E84,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" t="str">
-        <f>IF(Library!G85,Library!B85,"")</f>
-        <v/>
-      </c>
-      <c r="B77" t="str">
-        <f>IF(Library!G85,Library!D85,"")</f>
-        <v/>
-      </c>
-      <c r="C77" t="str">
-        <f>IF(Library!G85,CONCATENATE("barcode",TEXT(Library!C85,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D77" t="str">
-        <f>IF(AND(Library!G85,NOT(ISBLANK(Library!E85))),Library!E85,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" t="str">
-        <f>IF(Library!G86,Library!B86,"")</f>
-        <v/>
-      </c>
-      <c r="B78" t="str">
-        <f>IF(Library!G86,Library!D86,"")</f>
-        <v/>
-      </c>
-      <c r="C78" t="str">
-        <f>IF(Library!G86,CONCATENATE("barcode",TEXT(Library!C86,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D78" t="str">
-        <f>IF(AND(Library!G86,NOT(ISBLANK(Library!E86))),Library!E86,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" t="str">
-        <f>IF(Library!G87,Library!B87,"")</f>
-        <v/>
-      </c>
-      <c r="B79" t="str">
-        <f>IF(Library!G87,Library!D87,"")</f>
-        <v/>
-      </c>
-      <c r="C79" t="str">
-        <f>IF(Library!G87,CONCATENATE("barcode",TEXT(Library!C87,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D79" t="str">
-        <f>IF(AND(Library!G87,NOT(ISBLANK(Library!E87))),Library!E87,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" t="str">
-        <f>IF(Library!G88,Library!B88,"")</f>
-        <v/>
-      </c>
-      <c r="B80" t="str">
-        <f>IF(Library!G88,Library!D88,"")</f>
-        <v/>
-      </c>
-      <c r="C80" t="str">
-        <f>IF(Library!G88,CONCATENATE("barcode",TEXT(Library!C88,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D80" t="str">
-        <f>IF(AND(Library!G88,NOT(ISBLANK(Library!E88))),Library!E88,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" t="str">
-        <f>IF(Library!G89,Library!B89,"")</f>
-        <v/>
-      </c>
-      <c r="B81" t="str">
-        <f>IF(Library!G89,Library!D89,"")</f>
-        <v/>
-      </c>
-      <c r="C81" t="str">
-        <f>IF(Library!G89,CONCATENATE("barcode",TEXT(Library!C89,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D81" t="str">
-        <f>IF(AND(Library!G89,NOT(ISBLANK(Library!E89))),Library!E89,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" t="str">
-        <f>IF(Library!G90,Library!B90,"")</f>
-        <v/>
-      </c>
-      <c r="B82" t="str">
-        <f>IF(Library!G90,Library!D90,"")</f>
-        <v/>
-      </c>
-      <c r="C82" t="str">
-        <f>IF(Library!G90,CONCATENATE("barcode",TEXT(Library!C90,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D82" t="str">
-        <f>IF(AND(Library!G90,NOT(ISBLANK(Library!E90))),Library!E90,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" t="str">
-        <f>IF(Library!G91,Library!B91,"")</f>
-        <v/>
-      </c>
-      <c r="B83" t="str">
-        <f>IF(Library!G91,Library!D91,"")</f>
-        <v/>
-      </c>
-      <c r="C83" t="str">
-        <f>IF(Library!G91,CONCATENATE("barcode",TEXT(Library!C91,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D83" t="str">
-        <f>IF(AND(Library!G91,NOT(ISBLANK(Library!E91))),Library!E91,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" t="str">
-        <f>IF(Library!G92,Library!B92,"")</f>
-        <v/>
-      </c>
-      <c r="B84" t="str">
-        <f>IF(Library!G92,Library!D92,"")</f>
-        <v/>
-      </c>
-      <c r="C84" t="str">
-        <f>IF(Library!G92,CONCATENATE("barcode",TEXT(Library!C92,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D84" t="str">
-        <f>IF(AND(Library!G92,NOT(ISBLANK(Library!E92))),Library!E92,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" t="str">
-        <f>IF(Library!G93,Library!B93,"")</f>
-        <v/>
-      </c>
-      <c r="B85" t="str">
-        <f>IF(Library!G93,Library!D93,"")</f>
-        <v/>
-      </c>
-      <c r="C85" t="str">
-        <f>IF(Library!G93,CONCATENATE("barcode",TEXT(Library!C93,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D85" t="str">
-        <f>IF(AND(Library!G93,NOT(ISBLANK(Library!E93))),Library!E93,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" t="str">
-        <f>IF(Library!G94,Library!B94,"")</f>
-        <v/>
-      </c>
-      <c r="B86" t="str">
-        <f>IF(Library!G94,Library!D94,"")</f>
-        <v/>
-      </c>
-      <c r="C86" t="str">
-        <f>IF(Library!G94,CONCATENATE("barcode",TEXT(Library!C94,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D86" t="str">
-        <f>IF(AND(Library!G94,NOT(ISBLANK(Library!E94))),Library!E94,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" t="str">
-        <f>IF(Library!G95,Library!B95,"")</f>
-        <v/>
-      </c>
-      <c r="B87" t="str">
-        <f>IF(Library!G95,Library!D95,"")</f>
-        <v/>
-      </c>
-      <c r="C87" t="str">
-        <f>IF(Library!G95,CONCATENATE("barcode",TEXT(Library!C95,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D87" t="str">
-        <f>IF(AND(Library!G95,NOT(ISBLANK(Library!E95))),Library!E95,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" t="str">
-        <f>IF(Library!G96,Library!B96,"")</f>
-        <v/>
-      </c>
-      <c r="B88" t="str">
-        <f>IF(Library!G96,Library!D96,"")</f>
-        <v/>
-      </c>
-      <c r="C88" t="str">
-        <f>IF(Library!G96,CONCATENATE("barcode",TEXT(Library!C96,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D88" t="str">
-        <f>IF(AND(Library!G96,NOT(ISBLANK(Library!E96))),Library!E96,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" t="str">
-        <f>IF(Library!G97,Library!B97,"")</f>
-        <v/>
-      </c>
-      <c r="B89" t="str">
-        <f>IF(Library!G97,Library!D97,"")</f>
-        <v/>
-      </c>
-      <c r="C89" t="str">
-        <f>IF(Library!G97,CONCATENATE("barcode",TEXT(Library!C97,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D89" t="str">
-        <f>IF(AND(Library!G97,NOT(ISBLANK(Library!E97))),Library!E97,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" t="str">
-        <f>IF(Library!G98,Library!B98,"")</f>
-        <v/>
-      </c>
-      <c r="B90" t="str">
-        <f>IF(Library!G98,Library!D98,"")</f>
-        <v/>
-      </c>
-      <c r="C90" t="str">
-        <f>IF(Library!G98,CONCATENATE("barcode",TEXT(Library!C98,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D90" t="str">
-        <f>IF(AND(Library!G98,NOT(ISBLANK(Library!E98))),Library!E98,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" t="str">
-        <f>IF(Library!G99,Library!B99,"")</f>
-        <v/>
-      </c>
-      <c r="B91" t="str">
-        <f>IF(Library!G99,Library!D99,"")</f>
-        <v/>
-      </c>
-      <c r="C91" t="str">
-        <f>IF(Library!G99,CONCATENATE("barcode",TEXT(Library!C99,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D91" t="str">
-        <f>IF(AND(Library!G99,NOT(ISBLANK(Library!E99))),Library!E99,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" t="str">
-        <f>IF(Library!G100,Library!B100,"")</f>
-        <v/>
-      </c>
-      <c r="B92" t="str">
-        <f>IF(Library!G100,Library!D100,"")</f>
-        <v/>
-      </c>
-      <c r="C92" t="str">
-        <f>IF(Library!G100,CONCATENATE("barcode",TEXT(Library!C100,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D92" t="str">
-        <f>IF(AND(Library!G100,NOT(ISBLANK(Library!E100))),Library!E100,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" t="str">
-        <f>IF(Library!G101,Library!B101,"")</f>
-        <v/>
-      </c>
-      <c r="B93" t="str">
-        <f>IF(Library!G101,Library!D101,"")</f>
-        <v/>
-      </c>
-      <c r="C93" t="str">
-        <f>IF(Library!G101,CONCATENATE("barcode",TEXT(Library!C101,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D93" t="str">
-        <f>IF(AND(Library!G101,NOT(ISBLANK(Library!E101))),Library!E101,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" t="str">
-        <f>IF(Library!G102,Library!B102,"")</f>
-        <v/>
-      </c>
-      <c r="B94" t="str">
-        <f>IF(Library!G102,Library!D102,"")</f>
-        <v/>
-      </c>
-      <c r="C94" t="str">
-        <f>IF(Library!G102,CONCATENATE("barcode",TEXT(Library!C102,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D94" t="str">
-        <f>IF(AND(Library!G102,NOT(ISBLANK(Library!E102))),Library!E102,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" t="str">
-        <f>IF(Library!G103,Library!B103,"")</f>
-        <v/>
-      </c>
-      <c r="B95" t="str">
-        <f>IF(Library!G103,Library!D103,"")</f>
-        <v/>
-      </c>
-      <c r="C95" t="str">
-        <f>IF(Library!G103,CONCATENATE("barcode",TEXT(Library!C103,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D95" t="str">
-        <f>IF(AND(Library!G103,NOT(ISBLANK(Library!E103))),Library!E103,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" t="str">
-        <f>IF(Library!G104,Library!B104,"")</f>
-        <v/>
-      </c>
-      <c r="B96" t="str">
-        <f>IF(Library!G104,Library!D104,"")</f>
-        <v/>
-      </c>
-      <c r="C96" t="str">
-        <f>IF(Library!G104,CONCATENATE("barcode",TEXT(Library!C104,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D96" t="str">
-        <f>IF(AND(Library!G104,NOT(ISBLANK(Library!E104))),Library!E104,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" t="str">
-        <f>IF(Library!G105,Library!B105,"")</f>
-        <v/>
-      </c>
-      <c r="B97" t="str">
-        <f>IF(Library!G105,Library!D105,"")</f>
-        <v/>
-      </c>
-      <c r="C97" t="str">
-        <f>IF(Library!G105,CONCATENATE("barcode",TEXT(Library!C105,"00")),"")</f>
-        <v/>
-      </c>
-      <c r="D97" t="str">
-        <f>IF(AND(Library!G105,NOT(ISBLANK(Library!E105))),Library!E105,"")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="1Q6N0maAQNsOI43ZphZysMjsUMzPkWBybftcWP13tFYa3VpBIfjcO8oiJJC9/lEFsqnXug4WFdsAEbNVHfb6MQ==" saltValue="Li18yf8ME53aby/AQ6q8Qw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5817B840-46A1-4DBD-A947-D1215FFA570B}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
@@ -6464,7 +4659,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B1">
         <v>15</v>
@@ -6472,22 +4667,22 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -6496,7 +4691,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3BF958-2118-44FE-A2A7-C593F394324C}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
@@ -6509,17 +4704,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="16" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="16" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.4">
@@ -6527,42 +4722,42 @@
     </row>
     <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="18" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="109.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="16" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="168.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed sample types to pos/neg/field
</commit_message>
<xml_diff>
--- a/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
+++ b/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\git\nomadic\src\nomadic\start\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4A8232-E2E3-4D4E-9B71-C4B2CF93D9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{034844BD-1FC6-4103-939E-13D88771D5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="46260" windowHeight="23220" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="23292" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="2" r:id="rId1"/>
@@ -378,15 +378,6 @@
     <t>Post PCR DNA threshold (ng / µl)</t>
   </si>
   <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>Positive</t>
-  </si>
-  <si>
-    <t>Negative</t>
-  </si>
-  <si>
     <t>Barcode</t>
   </si>
   <si>
@@ -475,6 +466,15 @@
   </si>
   <si>
     <t>(auto-generated name to save this file as)</t>
+  </si>
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>pos</t>
+  </si>
+  <si>
+    <t>neg</t>
   </si>
 </sst>
 </file>
@@ -943,20 +943,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -969,9 +956,22 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1753,25 +1753,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
-        <v>126</v>
-      </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="A2" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" s="38"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
       <c r="E2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1780,67 +1780,67 @@
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
       <c r="E3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
       <c r="E4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="38" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
       <c r="E6" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="42" t="str">
+      <c r="B7" s="43"/>
+      <c r="C7" s="46" t="str">
         <f>IF(OR(ISBLANK(C2),ISBLANK(C3),ISBLANK(C4), ISBLANK(C5), ISBLANK(C6)),"",CONCATENATE(C2,"_",C3,TEXT(C5,"000"),"_",C4,"_Batch",C6))</f>
         <v/>
       </c>
-      <c r="D7" s="42"/>
+      <c r="D7" s="46"/>
       <c r="E7" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -1857,7 +1857,7 @@
         <v>105</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>102</v>
@@ -1866,16 +1866,16 @@
         <v>3</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -4583,6 +4583,12 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:I1"/>
@@ -4590,12 +4596,6 @@
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="B10:E105">
@@ -6442,7 +6442,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="1Q6N0maAQNsOI43ZphZysMjsUMzPkWBybftcWP13tFYa3VpBIfjcO8oiJJC9/lEFsqnXug4WFdsAEbNVHfb6MQ==" saltValue="Li18yf8ME53aby/AQ6q8Qw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="CfnnoxDcAKHMJC6Y5jSTtC6yVpOck4puJ4tDNPF6Iezid4asSt186XjyQmQrYinuLpTOZYY8Zm5No3k8dJcygw==" saltValue="nZxNFngO7dA1EOFhdWVH+A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
@@ -6477,21 +6477,21 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="dUxG8sZFHxMw0NDzxsm+4RagZS4zB7XJW9ODqWY1r6qy6zd7Iuke/o94IqDpwwU1NdNkvme+sj732vKg/zGkSg==" saltValue="+pMpwnpw0cbJIb7UlDcFSg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="xmn9xsOQyGD5/maqdLRhWCDyEicwLtiS1RammiH+O+XoHXEleFk1ZdTfkZwdA9/aPR5RrlKTYUBUKdzsCq/y+Q==" saltValue="uhLRvClRCRleXoflZ/4ABg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6509,17 +6509,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="16" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="16" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.4">
@@ -6527,42 +6527,42 @@
     </row>
     <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="18" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="109.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="16" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="168.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Changed sample types to pos/neg/field"
This reverts commit 3da3dea743255d7cd6588428c14392df9642be14.
</commit_message>
<xml_diff>
--- a/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
+++ b/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\git\nomadic\src\nomadic\start\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{034844BD-1FC6-4103-939E-13D88771D5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4A8232-E2E3-4D4E-9B71-C4B2CF93D9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="23292" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="46260" windowHeight="23220" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="2" r:id="rId1"/>
@@ -378,6 +378,15 @@
     <t>Post PCR DNA threshold (ng / µl)</t>
   </si>
   <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
     <t>Barcode</t>
   </si>
   <si>
@@ -466,15 +475,6 @@
   </si>
   <si>
     <t>(auto-generated name to save this file as)</t>
-  </si>
-  <si>
-    <t>field</t>
-  </si>
-  <si>
-    <t>pos</t>
-  </si>
-  <si>
-    <t>neg</t>
   </si>
 </sst>
 </file>
@@ -943,7 +943,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -956,22 +969,9 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1753,25 +1753,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
+      <c r="A2" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="40"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
       <c r="E2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1780,67 +1780,67 @@
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="40" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
       <c r="E4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
+      <c r="A5" s="40" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="40"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
       <c r="E5" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="42" t="s">
+      <c r="A6" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
       <c r="E6" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="46" t="str">
+      <c r="B7" s="39"/>
+      <c r="C7" s="42" t="str">
         <f>IF(OR(ISBLANK(C2),ISBLANK(C3),ISBLANK(C4), ISBLANK(C5), ISBLANK(C6)),"",CONCATENATE(C2,"_",C3,TEXT(C5,"000"),"_",C4,"_Batch",C6))</f>
         <v/>
       </c>
-      <c r="D7" s="46"/>
+      <c r="D7" s="42"/>
       <c r="E7" s="5" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -1857,7 +1857,7 @@
         <v>105</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>102</v>
@@ -1866,16 +1866,16 @@
         <v>3</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H9" s="28" t="s">
+        <v>135</v>
+      </c>
+      <c r="I9" s="29" t="s">
         <v>132</v>
-      </c>
-      <c r="I9" s="29" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -4583,12 +4583,6 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:I1"/>
@@ -4596,6 +4590,12 @@
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="B10:E105">
@@ -6442,7 +6442,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="CfnnoxDcAKHMJC6Y5jSTtC6yVpOck4puJ4tDNPF6Iezid4asSt186XjyQmQrYinuLpTOZYY8Zm5No3k8dJcygw==" saltValue="nZxNFngO7dA1EOFhdWVH+A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="1Q6N0maAQNsOI43ZphZysMjsUMzPkWBybftcWP13tFYa3VpBIfjcO8oiJJC9/lEFsqnXug4WFdsAEbNVHfb6MQ==" saltValue="Li18yf8ME53aby/AQ6q8Qw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
@@ -6477,21 +6477,21 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="xmn9xsOQyGD5/maqdLRhWCDyEicwLtiS1RammiH+O+XoHXEleFk1ZdTfkZwdA9/aPR5RrlKTYUBUKdzsCq/y+Q==" saltValue="uhLRvClRCRleXoflZ/4ABg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="dUxG8sZFHxMw0NDzxsm+4RagZS4zB7XJW9ODqWY1r6qy6zd7Iuke/o94IqDpwwU1NdNkvme+sj732vKg/zGkSg==" saltValue="+pMpwnpw0cbJIb7UlDcFSg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6509,17 +6509,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A2" s="16" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="16" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.4">
@@ -6527,42 +6527,42 @@
     </row>
     <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="109.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="168.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="16" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added substitute to geenrate correct sample_type names
</commit_message>
<xml_diff>
--- a/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
+++ b/src/nomadic/start/data/NOMADS_Library_Worksheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\git\nomadic\src\nomadic\start\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4A8232-E2E3-4D4E-9B71-C4B2CF93D9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D255FA76-F4E0-4A9D-914E-586C5B55DE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="46260" windowHeight="23220" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="23292" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="141">
   <si>
     <t>(YYYY-MM-DD)</t>
   </si>
@@ -475,6 +475,18 @@
   </si>
   <si>
     <t>(auto-generated name to save this file as)</t>
+  </si>
+  <si>
+    <t>nomadic_type</t>
+  </si>
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>pos</t>
+  </si>
+  <si>
+    <t>neg</t>
   </si>
 </sst>
 </file>
@@ -943,20 +955,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -969,9 +968,22 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -983,6 +995,9 @@
     <cellStyle name="Normal 4" xfId="5" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
   </cellStyles>
   <dxfs count="21">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1027,9 +1042,6 @@
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1546,13 +1558,13 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="sample_id">
       <calculatedColumnFormula>IF(Library!G10,Library!B10,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{98E62512-61AC-41C9-8930-37E9E6964CA3}" name="sample_type" dataDxfId="8">
-      <calculatedColumnFormula>IF(Library!G10,Library!D10,"")</calculatedColumnFormula>
+    <tableColumn id="9" xr3:uid="{98E62512-61AC-41C9-8930-37E9E6964CA3}" name="sample_type" dataDxfId="0">
+      <calculatedColumnFormula>IF(Library!G10,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D10,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="barcode" dataDxfId="7">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="barcode" dataDxfId="8">
       <calculatedColumnFormula>IF(Library!G10,CONCATENATE("barcode",TEXT(Library!C10,"00")),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1FDA51E1-A0B8-4EA2-9C5A-4746ACED2260}" name="post_pcr_dna_conc_ngul" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{1FDA51E1-A0B8-4EA2-9C5A-4746ACED2260}" name="post_pcr_dna_conc_ngul" dataDxfId="7">
       <calculatedColumnFormula>IF(AND(Library!G10,NOT(ISBLANK(Library!E10))),Library!E10,"")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1753,25 +1765,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="38" t="s">
         <v>126</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
       <c r="E2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1780,34 +1792,34 @@
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
       <c r="E3" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
       <c r="E4" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="6" t="s">
         <v>129</v>
       </c>
@@ -1816,12 +1828,12 @@
       <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
       <c r="E6" s="5" t="s">
         <v>125</v>
       </c>
@@ -1830,15 +1842,15 @@
       <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="42" t="str">
+      <c r="B7" s="43"/>
+      <c r="C7" s="46" t="str">
         <f>IF(OR(ISBLANK(C2),ISBLANK(C3),ISBLANK(C4), ISBLANK(C5), ISBLANK(C6)),"",CONCATENATE(C2,"_",C3,TEXT(C5,"000"),"_",C4,"_Batch",C6))</f>
         <v/>
       </c>
-      <c r="D7" s="42"/>
+      <c r="D7" s="46"/>
       <c r="E7" s="5" t="s">
         <v>136</v>
       </c>
@@ -4583,6 +4595,12 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="13">
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:I1"/>
@@ -4590,38 +4608,32 @@
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="B10:E105">
-    <cfRule type="expression" dxfId="5" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="6" priority="5" stopIfTrue="1">
       <formula>COUNTIF(B10,"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C6">
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>COUNTIF(C2,"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10:C105">
-    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E105">
-    <cfRule type="cellIs" dxfId="2" priority="9" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="between">
       <formula>0</formula>
       <formula>Post_PCR_DNA_threshold_ngul</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="10" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="2" priority="10" operator="greaterThanOrEqual">
       <formula>Post_PCR_DNA_threshold_ngul</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:I105">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>NOT(COUNTIF(I10,""))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4719,7 +4731,7 @@
         <v/>
       </c>
       <c r="B2" t="str">
-        <f>IF(Library!G10,Library!D10,"")</f>
+        <f>IF(Library!G10,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D10,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C2" t="str">
@@ -4737,7 +4749,7 @@
         <v/>
       </c>
       <c r="B3" t="str">
-        <f>IF(Library!G11,Library!D11,"")</f>
+        <f>IF(Library!G11,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D11,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C3" t="str">
@@ -4755,7 +4767,7 @@
         <v/>
       </c>
       <c r="B4" t="str">
-        <f>IF(Library!G12,Library!D12,"")</f>
+        <f>IF(Library!G12,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D12,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C4" t="str">
@@ -4773,7 +4785,7 @@
         <v/>
       </c>
       <c r="B5" t="str">
-        <f>IF(Library!G13,Library!D13,"")</f>
+        <f>IF(Library!G13,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D13,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C5" t="str">
@@ -4791,7 +4803,7 @@
         <v/>
       </c>
       <c r="B6" t="str">
-        <f>IF(Library!G14,Library!D14,"")</f>
+        <f>IF(Library!G14,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D14,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C6" t="str">
@@ -4809,7 +4821,7 @@
         <v/>
       </c>
       <c r="B7" t="str">
-        <f>IF(Library!G15,Library!D15,"")</f>
+        <f>IF(Library!G15,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D15,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C7" t="str">
@@ -4827,7 +4839,7 @@
         <v/>
       </c>
       <c r="B8" t="str">
-        <f>IF(Library!G16,Library!D16,"")</f>
+        <f>IF(Library!G16,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D16,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C8" t="str">
@@ -4845,7 +4857,7 @@
         <v/>
       </c>
       <c r="B9" t="str">
-        <f>IF(Library!G17,Library!D17,"")</f>
+        <f>IF(Library!G17,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D17,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C9" t="str">
@@ -4863,7 +4875,7 @@
         <v/>
       </c>
       <c r="B10" t="str">
-        <f>IF(Library!G18,Library!D18,"")</f>
+        <f>IF(Library!G18,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D18,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C10" t="str">
@@ -4881,7 +4893,7 @@
         <v/>
       </c>
       <c r="B11" t="str">
-        <f>IF(Library!G19,Library!D19,"")</f>
+        <f>IF(Library!G19,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D19,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C11" t="str">
@@ -4899,7 +4911,7 @@
         <v/>
       </c>
       <c r="B12" t="str">
-        <f>IF(Library!G20,Library!D20,"")</f>
+        <f>IF(Library!G20,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D20,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C12" t="str">
@@ -4917,7 +4929,7 @@
         <v/>
       </c>
       <c r="B13" t="str">
-        <f>IF(Library!G21,Library!D21,"")</f>
+        <f>IF(Library!G21,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D21,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C13" t="str">
@@ -4935,7 +4947,7 @@
         <v/>
       </c>
       <c r="B14" t="str">
-        <f>IF(Library!G22,Library!D22,"")</f>
+        <f>IF(Library!G22,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D22,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C14" t="str">
@@ -4953,7 +4965,7 @@
         <v/>
       </c>
       <c r="B15" t="str">
-        <f>IF(Library!G23,Library!D23,"")</f>
+        <f>IF(Library!G23,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D23,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C15" t="str">
@@ -4971,7 +4983,7 @@
         <v/>
       </c>
       <c r="B16" t="str">
-        <f>IF(Library!G24,Library!D24,"")</f>
+        <f>IF(Library!G24,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D24,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C16" t="str">
@@ -4989,7 +5001,7 @@
         <v/>
       </c>
       <c r="B17" t="str">
-        <f>IF(Library!G25,Library!D25,"")</f>
+        <f>IF(Library!G25,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D25,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C17" t="str">
@@ -5007,7 +5019,7 @@
         <v/>
       </c>
       <c r="B18" t="str">
-        <f>IF(Library!G26,Library!D26,"")</f>
+        <f>IF(Library!G26,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D26,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C18" t="str">
@@ -5025,7 +5037,7 @@
         <v/>
       </c>
       <c r="B19" t="str">
-        <f>IF(Library!G27,Library!D27,"")</f>
+        <f>IF(Library!G27,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D27,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C19" t="str">
@@ -5043,7 +5055,7 @@
         <v/>
       </c>
       <c r="B20" t="str">
-        <f>IF(Library!G28,Library!D28,"")</f>
+        <f>IF(Library!G28,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D28,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C20" t="str">
@@ -5061,7 +5073,7 @@
         <v/>
       </c>
       <c r="B21" t="str">
-        <f>IF(Library!G29,Library!D29,"")</f>
+        <f>IF(Library!G29,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D29,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C21" t="str">
@@ -5079,7 +5091,7 @@
         <v/>
       </c>
       <c r="B22" t="str">
-        <f>IF(Library!G30,Library!D30,"")</f>
+        <f>IF(Library!G30,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D30,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C22" t="str">
@@ -5097,7 +5109,7 @@
         <v/>
       </c>
       <c r="B23" t="str">
-        <f>IF(Library!G31,Library!D31,"")</f>
+        <f>IF(Library!G31,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D31,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C23" t="str">
@@ -5115,7 +5127,7 @@
         <v/>
       </c>
       <c r="B24" t="str">
-        <f>IF(Library!G32,Library!D32,"")</f>
+        <f>IF(Library!G32,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D32,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C24" t="str">
@@ -5133,7 +5145,7 @@
         <v/>
       </c>
       <c r="B25" t="str">
-        <f>IF(Library!G33,Library!D33,"")</f>
+        <f>IF(Library!G33,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D33,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C25" t="str">
@@ -5151,7 +5163,7 @@
         <v/>
       </c>
       <c r="B26" t="str">
-        <f>IF(Library!G34,Library!D34,"")</f>
+        <f>IF(Library!G34,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D34,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C26" t="str">
@@ -5169,7 +5181,7 @@
         <v/>
       </c>
       <c r="B27" t="str">
-        <f>IF(Library!G35,Library!D35,"")</f>
+        <f>IF(Library!G35,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D35,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C27" t="str">
@@ -5187,7 +5199,7 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <f>IF(Library!G36,Library!D36,"")</f>
+        <f>IF(Library!G36,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D36,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C28" t="str">
@@ -5205,7 +5217,7 @@
         <v/>
       </c>
       <c r="B29" t="str">
-        <f>IF(Library!G37,Library!D37,"")</f>
+        <f>IF(Library!G37,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D37,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C29" t="str">
@@ -5223,7 +5235,7 @@
         <v/>
       </c>
       <c r="B30" t="str">
-        <f>IF(Library!G38,Library!D38,"")</f>
+        <f>IF(Library!G38,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D38,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C30" t="str">
@@ -5241,7 +5253,7 @@
         <v/>
       </c>
       <c r="B31" t="str">
-        <f>IF(Library!G39,Library!D39,"")</f>
+        <f>IF(Library!G39,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D39,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C31" t="str">
@@ -5259,7 +5271,7 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <f>IF(Library!G40,Library!D40,"")</f>
+        <f>IF(Library!G40,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D40,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C32" t="str">
@@ -5277,7 +5289,7 @@
         <v/>
       </c>
       <c r="B33" t="str">
-        <f>IF(Library!G41,Library!D41,"")</f>
+        <f>IF(Library!G41,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D41,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C33" t="str">
@@ -5295,7 +5307,7 @@
         <v/>
       </c>
       <c r="B34" t="str">
-        <f>IF(Library!G42,Library!D42,"")</f>
+        <f>IF(Library!G42,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D42,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C34" t="str">
@@ -5313,7 +5325,7 @@
         <v/>
       </c>
       <c r="B35" t="str">
-        <f>IF(Library!G43,Library!D43,"")</f>
+        <f>IF(Library!G43,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D43,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C35" t="str">
@@ -5331,7 +5343,7 @@
         <v/>
       </c>
       <c r="B36" t="str">
-        <f>IF(Library!G44,Library!D44,"")</f>
+        <f>IF(Library!G44,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D44,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C36" t="str">
@@ -5349,7 +5361,7 @@
         <v/>
       </c>
       <c r="B37" t="str">
-        <f>IF(Library!G45,Library!D45,"")</f>
+        <f>IF(Library!G45,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D45,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C37" t="str">
@@ -5367,7 +5379,7 @@
         <v/>
       </c>
       <c r="B38" t="str">
-        <f>IF(Library!G46,Library!D46,"")</f>
+        <f>IF(Library!G46,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D46,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C38" t="str">
@@ -5385,7 +5397,7 @@
         <v/>
       </c>
       <c r="B39" t="str">
-        <f>IF(Library!G47,Library!D47,"")</f>
+        <f>IF(Library!G47,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D47,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C39" t="str">
@@ -5403,7 +5415,7 @@
         <v/>
       </c>
       <c r="B40" t="str">
-        <f>IF(Library!G48,Library!D48,"")</f>
+        <f>IF(Library!G48,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D48,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C40" t="str">
@@ -5421,7 +5433,7 @@
         <v/>
       </c>
       <c r="B41" t="str">
-        <f>IF(Library!G49,Library!D49,"")</f>
+        <f>IF(Library!G49,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D49,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C41" t="str">
@@ -5439,7 +5451,7 @@
         <v/>
       </c>
       <c r="B42" t="str">
-        <f>IF(Library!G50,Library!D50,"")</f>
+        <f>IF(Library!G50,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D50,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C42" t="str">
@@ -5457,7 +5469,7 @@
         <v/>
       </c>
       <c r="B43" t="str">
-        <f>IF(Library!G51,Library!D51,"")</f>
+        <f>IF(Library!G51,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D51,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C43" t="str">
@@ -5475,7 +5487,7 @@
         <v/>
       </c>
       <c r="B44" t="str">
-        <f>IF(Library!G52,Library!D52,"")</f>
+        <f>IF(Library!G52,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D52,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C44" t="str">
@@ -5493,7 +5505,7 @@
         <v/>
       </c>
       <c r="B45" t="str">
-        <f>IF(Library!G53,Library!D53,"")</f>
+        <f>IF(Library!G53,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D53,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C45" t="str">
@@ -5511,7 +5523,7 @@
         <v/>
       </c>
       <c r="B46" t="str">
-        <f>IF(Library!G54,Library!D54,"")</f>
+        <f>IF(Library!G54,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D54,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C46" t="str">
@@ -5529,7 +5541,7 @@
         <v/>
       </c>
       <c r="B47" t="str">
-        <f>IF(Library!G55,Library!D55,"")</f>
+        <f>IF(Library!G55,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D55,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C47" t="str">
@@ -5547,7 +5559,7 @@
         <v/>
       </c>
       <c r="B48" t="str">
-        <f>IF(Library!G56,Library!D56,"")</f>
+        <f>IF(Library!G56,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D56,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C48" t="str">
@@ -5565,7 +5577,7 @@
         <v/>
       </c>
       <c r="B49" t="str">
-        <f>IF(Library!G57,Library!D57,"")</f>
+        <f>IF(Library!G57,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D57,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C49" t="str">
@@ -5583,7 +5595,7 @@
         <v/>
       </c>
       <c r="B50" t="str">
-        <f>IF(Library!G58,Library!D58,"")</f>
+        <f>IF(Library!G58,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D58,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C50" t="str">
@@ -5601,7 +5613,7 @@
         <v/>
       </c>
       <c r="B51" t="str">
-        <f>IF(Library!G59,Library!D59,"")</f>
+        <f>IF(Library!G59,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D59,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C51" t="str">
@@ -5619,7 +5631,7 @@
         <v/>
       </c>
       <c r="B52" t="str">
-        <f>IF(Library!G60,Library!D60,"")</f>
+        <f>IF(Library!G60,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D60,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C52" t="str">
@@ -5637,7 +5649,7 @@
         <v/>
       </c>
       <c r="B53" t="str">
-        <f>IF(Library!G61,Library!D61,"")</f>
+        <f>IF(Library!G61,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D61,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C53" t="str">
@@ -5655,7 +5667,7 @@
         <v/>
       </c>
       <c r="B54" t="str">
-        <f>IF(Library!G62,Library!D62,"")</f>
+        <f>IF(Library!G62,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D62,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C54" t="str">
@@ -5673,7 +5685,7 @@
         <v/>
       </c>
       <c r="B55" t="str">
-        <f>IF(Library!G63,Library!D63,"")</f>
+        <f>IF(Library!G63,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D63,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C55" t="str">
@@ -5691,7 +5703,7 @@
         <v/>
       </c>
       <c r="B56" t="str">
-        <f>IF(Library!G64,Library!D64,"")</f>
+        <f>IF(Library!G64,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D64,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C56" t="str">
@@ -5709,7 +5721,7 @@
         <v/>
       </c>
       <c r="B57" t="str">
-        <f>IF(Library!G65,Library!D65,"")</f>
+        <f>IF(Library!G65,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D65,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C57" t="str">
@@ -5727,7 +5739,7 @@
         <v/>
       </c>
       <c r="B58" t="str">
-        <f>IF(Library!G66,Library!D66,"")</f>
+        <f>IF(Library!G66,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D66,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C58" t="str">
@@ -5745,7 +5757,7 @@
         <v/>
       </c>
       <c r="B59" t="str">
-        <f>IF(Library!G67,Library!D67,"")</f>
+        <f>IF(Library!G67,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D67,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C59" t="str">
@@ -5763,7 +5775,7 @@
         <v/>
       </c>
       <c r="B60" t="str">
-        <f>IF(Library!G68,Library!D68,"")</f>
+        <f>IF(Library!G68,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D68,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C60" t="str">
@@ -5781,7 +5793,7 @@
         <v/>
       </c>
       <c r="B61" t="str">
-        <f>IF(Library!G69,Library!D69,"")</f>
+        <f>IF(Library!G69,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D69,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C61" t="str">
@@ -5799,7 +5811,7 @@
         <v/>
       </c>
       <c r="B62" t="str">
-        <f>IF(Library!G70,Library!D70,"")</f>
+        <f>IF(Library!G70,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D70,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C62" t="str">
@@ -5817,7 +5829,7 @@
         <v/>
       </c>
       <c r="B63" t="str">
-        <f>IF(Library!G71,Library!D71,"")</f>
+        <f>IF(Library!G71,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D71,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C63" t="str">
@@ -5835,7 +5847,7 @@
         <v/>
       </c>
       <c r="B64" t="str">
-        <f>IF(Library!G72,Library!D72,"")</f>
+        <f>IF(Library!G72,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D72,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C64" t="str">
@@ -5853,7 +5865,7 @@
         <v/>
       </c>
       <c r="B65" t="str">
-        <f>IF(Library!G73,Library!D73,"")</f>
+        <f>IF(Library!G73,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D73,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C65" t="str">
@@ -5871,7 +5883,7 @@
         <v/>
       </c>
       <c r="B66" t="str">
-        <f>IF(Library!G74,Library!D74,"")</f>
+        <f>IF(Library!G74,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D74,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C66" t="str">
@@ -5889,7 +5901,7 @@
         <v/>
       </c>
       <c r="B67" t="str">
-        <f>IF(Library!G75,Library!D75,"")</f>
+        <f>IF(Library!G75,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D75,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C67" t="str">
@@ -5907,7 +5919,7 @@
         <v/>
       </c>
       <c r="B68" t="str">
-        <f>IF(Library!G76,Library!D76,"")</f>
+        <f>IF(Library!G76,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D76,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C68" t="str">
@@ -5925,7 +5937,7 @@
         <v/>
       </c>
       <c r="B69" t="str">
-        <f>IF(Library!G77,Library!D77,"")</f>
+        <f>IF(Library!G77,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D77,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C69" t="str">
@@ -5943,7 +5955,7 @@
         <v/>
       </c>
       <c r="B70" t="str">
-        <f>IF(Library!G78,Library!D78,"")</f>
+        <f>IF(Library!G78,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D78,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C70" t="str">
@@ -5961,7 +5973,7 @@
         <v/>
       </c>
       <c r="B71" t="str">
-        <f>IF(Library!G79,Library!D79,"")</f>
+        <f>IF(Library!G79,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D79,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C71" t="str">
@@ -5979,7 +5991,7 @@
         <v/>
       </c>
       <c r="B72" t="str">
-        <f>IF(Library!G80,Library!D80,"")</f>
+        <f>IF(Library!G80,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D80,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C72" t="str">
@@ -5997,7 +6009,7 @@
         <v/>
       </c>
       <c r="B73" t="str">
-        <f>IF(Library!G81,Library!D81,"")</f>
+        <f>IF(Library!G81,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D81,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C73" t="str">
@@ -6015,7 +6027,7 @@
         <v/>
       </c>
       <c r="B74" t="str">
-        <f>IF(Library!G82,Library!D82,"")</f>
+        <f>IF(Library!G82,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D82,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C74" t="str">
@@ -6033,7 +6045,7 @@
         <v/>
       </c>
       <c r="B75" t="str">
-        <f>IF(Library!G83,Library!D83,"")</f>
+        <f>IF(Library!G83,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D83,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C75" t="str">
@@ -6051,7 +6063,7 @@
         <v/>
       </c>
       <c r="B76" t="str">
-        <f>IF(Library!G84,Library!D84,"")</f>
+        <f>IF(Library!G84,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D84,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C76" t="str">
@@ -6069,7 +6081,7 @@
         <v/>
       </c>
       <c r="B77" t="str">
-        <f>IF(Library!G85,Library!D85,"")</f>
+        <f>IF(Library!G85,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D85,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C77" t="str">
@@ -6087,7 +6099,7 @@
         <v/>
       </c>
       <c r="B78" t="str">
-        <f>IF(Library!G86,Library!D86,"")</f>
+        <f>IF(Library!G86,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D86,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C78" t="str">
@@ -6105,7 +6117,7 @@
         <v/>
       </c>
       <c r="B79" t="str">
-        <f>IF(Library!G87,Library!D87,"")</f>
+        <f>IF(Library!G87,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D87,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C79" t="str">
@@ -6123,7 +6135,7 @@
         <v/>
       </c>
       <c r="B80" t="str">
-        <f>IF(Library!G88,Library!D88,"")</f>
+        <f>IF(Library!G88,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D88,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C80" t="str">
@@ -6141,7 +6153,7 @@
         <v/>
       </c>
       <c r="B81" t="str">
-        <f>IF(Library!G89,Library!D89,"")</f>
+        <f>IF(Library!G89,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D89,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C81" t="str">
@@ -6159,7 +6171,7 @@
         <v/>
       </c>
       <c r="B82" t="str">
-        <f>IF(Library!G90,Library!D90,"")</f>
+        <f>IF(Library!G90,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D90,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C82" t="str">
@@ -6177,7 +6189,7 @@
         <v/>
       </c>
       <c r="B83" t="str">
-        <f>IF(Library!G91,Library!D91,"")</f>
+        <f>IF(Library!G91,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D91,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C83" t="str">
@@ -6195,7 +6207,7 @@
         <v/>
       </c>
       <c r="B84" t="str">
-        <f>IF(Library!G92,Library!D92,"")</f>
+        <f>IF(Library!G92,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D92,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C84" t="str">
@@ -6213,7 +6225,7 @@
         <v/>
       </c>
       <c r="B85" t="str">
-        <f>IF(Library!G93,Library!D93,"")</f>
+        <f>IF(Library!G93,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D93,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C85" t="str">
@@ -6231,7 +6243,7 @@
         <v/>
       </c>
       <c r="B86" t="str">
-        <f>IF(Library!G94,Library!D94,"")</f>
+        <f>IF(Library!G94,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D94,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C86" t="str">
@@ -6249,7 +6261,7 @@
         <v/>
       </c>
       <c r="B87" t="str">
-        <f>IF(Library!G95,Library!D95,"")</f>
+        <f>IF(Library!G95,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D95,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C87" t="str">
@@ -6267,7 +6279,7 @@
         <v/>
       </c>
       <c r="B88" t="str">
-        <f>IF(Library!G96,Library!D96,"")</f>
+        <f>IF(Library!G96,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D96,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C88" t="str">
@@ -6285,7 +6297,7 @@
         <v/>
       </c>
       <c r="B89" t="str">
-        <f>IF(Library!G97,Library!D97,"")</f>
+        <f>IF(Library!G97,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D97,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C89" t="str">
@@ -6303,7 +6315,7 @@
         <v/>
       </c>
       <c r="B90" t="str">
-        <f>IF(Library!G98,Library!D98,"")</f>
+        <f>IF(Library!G98,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D98,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C90" t="str">
@@ -6321,7 +6333,7 @@
         <v/>
       </c>
       <c r="B91" t="str">
-        <f>IF(Library!G99,Library!D99,"")</f>
+        <f>IF(Library!G99,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D99,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C91" t="str">
@@ -6339,7 +6351,7 @@
         <v/>
       </c>
       <c r="B92" t="str">
-        <f>IF(Library!G100,Library!D100,"")</f>
+        <f>IF(Library!G100,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D100,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C92" t="str">
@@ -6357,7 +6369,7 @@
         <v/>
       </c>
       <c r="B93" t="str">
-        <f>IF(Library!G101,Library!D101,"")</f>
+        <f>IF(Library!G101,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D101,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C93" t="str">
@@ -6375,7 +6387,7 @@
         <v/>
       </c>
       <c r="B94" t="str">
-        <f>IF(Library!G102,Library!D102,"")</f>
+        <f>IF(Library!G102,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D102,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C94" t="str">
@@ -6393,7 +6405,7 @@
         <v/>
       </c>
       <c r="B95" t="str">
-        <f>IF(Library!G103,Library!D103,"")</f>
+        <f>IF(Library!G103,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D103,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C95" t="str">
@@ -6411,7 +6423,7 @@
         <v/>
       </c>
       <c r="B96" t="str">
-        <f>IF(Library!G104,Library!D104,"")</f>
+        <f>IF(Library!G104,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D104,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C96" t="str">
@@ -6429,7 +6441,7 @@
         <v/>
       </c>
       <c r="B97" t="str">
-        <f>IF(Library!G105,Library!D105,"")</f>
+        <f>IF(Library!G105,SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(Library!D105,options!$A$5,options!$B$5),options!$A$6,options!$B$6),options!$A$7,options!$B$7),"")</f>
         <v/>
       </c>
       <c r="C97" t="str">
@@ -6442,7 +6454,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="1Q6N0maAQNsOI43ZphZysMjsUMzPkWBybftcWP13tFYa3VpBIfjcO8oiJJC9/lEFsqnXug4WFdsAEbNVHfb6MQ==" saltValue="Li18yf8ME53aby/AQ6q8Qw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="1ybfLyjx3JNymf5UayvI8KwqN/GLJKMCjx5IXv1Zax162N0CTpn1sglGS5rATenleJOrXZWis5Bo6BFJ33fEsA==" saltValue="+RvCQ1wPJPQUirC2rcHswQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <tableParts count="1">
@@ -6459,7 +6471,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.09765625" customWidth="1"/>
+    <col min="1" max="1" width="29.5" customWidth="1"/>
+    <col min="2" max="2" width="24.3984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -6474,24 +6487,36 @@
       <c r="A4" s="12" t="s">
         <v>103</v>
       </c>
+      <c r="B4" s="12" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>111</v>
       </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>112</v>
       </c>
+      <c r="B6" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>113</v>
       </c>
+      <c r="B7" t="s">
+        <v>140</v>
+      </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="dUxG8sZFHxMw0NDzxsm+4RagZS4zB7XJW9ODqWY1r6qy6zd7Iuke/o94IqDpwwU1NdNkvme+sj732vKg/zGkSg==" saltValue="+pMpwnpw0cbJIb7UlDcFSg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="2jtMf6v2Bc0I3DUhZIQvGDdl0l6k2W0erOWmfVpGfXqnIih+xuwPX1D3EB0JYQvUtyxHtjnaGNil89tYVsO5YQ==" saltValue="SV1PjuSXPWz6AX0tsMJUSg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>